<commit_message>
Apply pending portal updates
</commit_message>
<xml_diff>
--- a/public/templates/ACSS Open Data Assesment Tools.xlsx
+++ b/public/templates/ACSS Open Data Assesment Tools.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8EFD1B9-886F-4624-84DA-C7EE72E4A2BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40532226-9DB3-4007-83CA-1161F6D83F45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="294">
   <si>
     <t>ACSS Open Data Assesment Tools</t>
   </si>
@@ -856,22 +856,6 @@
   </si>
   <si>
     <r>
-      <t>iii.     By Sector/ Activities</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>^</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">iv.     By Intra, Extra </t>
     </r>
     <r>
@@ -1718,6 +1702,27 @@
   </si>
   <si>
     <t>CN.RUS.FAP.000</t>
+  </si>
+  <si>
+    <t>CN.RUS.NRR.000</t>
+  </si>
+  <si>
+    <r>
+      <t>National Recycling Rate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (1)</t>
+    </r>
+  </si>
+  <si>
+    <t>iii.     By Sector/ Activities</t>
   </si>
 </sst>
 </file>
@@ -2406,7 +2411,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="23" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="127">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2653,20 +2658,53 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -2674,54 +2712,6 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="30" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -2746,17 +2736,48 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -2770,8 +2791,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF0000FF"/>
       <color rgb="FF00B0F0"/>
-      <color rgb="FF0000FF"/>
     </mruColors>
   </colors>
   <extLst>
@@ -3051,10 +3072,10 @@
   <sheetPr>
     <tabColor rgb="FF0070C0"/>
   </sheetPr>
-  <dimension ref="A1:U99"/>
+  <dimension ref="A1:U100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.140625" customWidth="1"/>
+    <col min="1" max="1" width="2.140625" style="114" customWidth="1"/>
     <col min="2" max="2" width="17.140625" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" customWidth="1"/>
     <col min="4" max="4" width="61.85546875" customWidth="1"/>
@@ -3083,11 +3104,11 @@
       </c>
     </row>
     <row r="2" spans="1:21" ht="40.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="98" t="s">
+      <c r="B2" s="96" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="99"/>
-      <c r="D2" s="99"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
       <c r="E2" s="18" t="s">
         <v>2</v>
       </c>
@@ -3096,64 +3117,64 @@
       </c>
     </row>
     <row r="3" spans="1:21" s="4" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="119" t="s">
-        <v>214</v>
-      </c>
-      <c r="B3" s="94" t="s">
+      <c r="A3" s="115" t="s">
+        <v>213</v>
+      </c>
+      <c r="B3" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="94" t="s">
+      <c r="C3" s="98" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="94" t="s">
+      <c r="D3" s="98" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="94" t="s">
+      <c r="E3" s="98" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="94" t="s">
+      <c r="F3" s="98" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="94" t="s">
+      <c r="G3" s="98" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="94" t="s">
+      <c r="H3" s="98" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="94" t="s">
+      <c r="I3" s="98" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="93" t="s">
+      <c r="J3" s="101" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="93"/>
-      <c r="L3" s="93"/>
-      <c r="M3" s="93"/>
-      <c r="N3" s="93" t="s">
+      <c r="K3" s="101"/>
+      <c r="L3" s="101"/>
+      <c r="M3" s="101"/>
+      <c r="N3" s="101" t="s">
         <v>12</v>
       </c>
-      <c r="O3" s="93"/>
-      <c r="P3" s="93"/>
-      <c r="Q3" s="93"/>
-      <c r="R3" s="93"/>
-      <c r="S3" s="93"/>
-      <c r="T3" s="94" t="s">
+      <c r="O3" s="101"/>
+      <c r="P3" s="101"/>
+      <c r="Q3" s="101"/>
+      <c r="R3" s="101"/>
+      <c r="S3" s="101"/>
+      <c r="T3" s="98" t="s">
         <v>13</v>
       </c>
-      <c r="U3" s="94" t="s">
+      <c r="U3" s="98" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:21" s="4" customFormat="1" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="119"/>
-      <c r="B4" s="94"/>
-      <c r="C4" s="94"/>
-      <c r="D4" s="94"/>
-      <c r="E4" s="94"/>
-      <c r="F4" s="94"/>
-      <c r="G4" s="94"/>
-      <c r="H4" s="94"/>
-      <c r="I4" s="94"/>
+      <c r="A4" s="115"/>
+      <c r="B4" s="98"/>
+      <c r="C4" s="98"/>
+      <c r="D4" s="98"/>
+      <c r="E4" s="98"/>
+      <c r="F4" s="98"/>
+      <c r="G4" s="98"/>
+      <c r="H4" s="98"/>
+      <c r="I4" s="98"/>
       <c r="J4" s="60" t="s">
         <v>15</v>
       </c>
@@ -3184,14 +3205,14 @@
       <c r="S4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="T4" s="94"/>
-      <c r="U4" s="94"/>
+      <c r="T4" s="98"/>
+      <c r="U4" s="98"/>
     </row>
     <row r="5" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="120" t="s">
-        <v>215</v>
-      </c>
-      <c r="B5" s="101" t="s">
+      <c r="A5" s="116" t="s">
+        <v>214</v>
+      </c>
+      <c r="B5" s="94" t="s">
         <v>25</v>
       </c>
       <c r="C5" s="95" t="s">
@@ -3260,10 +3281,10 @@
       <c r="U5" s="26"/>
     </row>
     <row r="6" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="120" t="s">
-        <v>216</v>
-      </c>
-      <c r="B6" s="101"/>
+      <c r="A6" s="116" t="s">
+        <v>215</v>
+      </c>
+      <c r="B6" s="94"/>
       <c r="C6" s="95"/>
       <c r="D6" s="95"/>
       <c r="E6" s="2" t="s">
@@ -3326,10 +3347,10 @@
       <c r="U6" s="26"/>
     </row>
     <row r="7" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="120" t="s">
-        <v>217</v>
-      </c>
-      <c r="B7" s="101"/>
+      <c r="A7" s="116" t="s">
+        <v>216</v>
+      </c>
+      <c r="B7" s="94"/>
       <c r="C7" s="95"/>
       <c r="D7" s="17" t="s">
         <v>30</v>
@@ -3394,10 +3415,10 @@
       <c r="U7" s="26"/>
     </row>
     <row r="8" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="120" t="s">
-        <v>218</v>
-      </c>
-      <c r="B8" s="101"/>
+      <c r="A8" s="116" t="s">
+        <v>217</v>
+      </c>
+      <c r="B8" s="94"/>
       <c r="C8" s="95"/>
       <c r="D8" s="17" t="s">
         <v>32</v>
@@ -3460,10 +3481,10 @@
       <c r="U8" s="26"/>
     </row>
     <row r="9" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="120" t="s">
-        <v>219</v>
-      </c>
-      <c r="B9" s="101"/>
+      <c r="A9" s="116" t="s">
+        <v>218</v>
+      </c>
+      <c r="B9" s="94"/>
       <c r="C9" s="95" t="s">
         <v>33</v>
       </c>
@@ -3528,10 +3549,10 @@
       <c r="U9" s="26"/>
     </row>
     <row r="10" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="120" t="s">
-        <v>220</v>
-      </c>
-      <c r="B10" s="101"/>
+      <c r="A10" s="116" t="s">
+        <v>219</v>
+      </c>
+      <c r="B10" s="94"/>
       <c r="C10" s="95"/>
       <c r="D10" s="95"/>
       <c r="E10" s="2" t="s">
@@ -3594,10 +3615,10 @@
       <c r="U10" s="26"/>
     </row>
     <row r="11" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="120" t="s">
-        <v>221</v>
-      </c>
-      <c r="B11" s="101"/>
+      <c r="A11" s="116" t="s">
+        <v>220</v>
+      </c>
+      <c r="B11" s="94"/>
       <c r="C11" s="95"/>
       <c r="D11" s="95"/>
       <c r="E11" s="2" t="s">
@@ -3660,10 +3681,10 @@
       <c r="U11" s="26"/>
     </row>
     <row r="12" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="120" t="s">
-        <v>222</v>
-      </c>
-      <c r="B12" s="101"/>
+      <c r="A12" s="116" t="s">
+        <v>221</v>
+      </c>
+      <c r="B12" s="94"/>
       <c r="C12" s="95"/>
       <c r="D12" s="95"/>
       <c r="E12" s="2" t="s">
@@ -3726,10 +3747,10 @@
       <c r="U12" s="26"/>
     </row>
     <row r="13" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="120" t="s">
-        <v>223</v>
-      </c>
-      <c r="B13" s="101"/>
+      <c r="A13" s="116" t="s">
+        <v>222</v>
+      </c>
+      <c r="B13" s="94"/>
       <c r="C13" s="95"/>
       <c r="D13" s="17" t="s">
         <v>37</v>
@@ -3792,10 +3813,10 @@
       <c r="U13" s="26"/>
     </row>
     <row r="14" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="120" t="s">
-        <v>224</v>
-      </c>
-      <c r="B14" s="101"/>
+      <c r="A14" s="116" t="s">
+        <v>223</v>
+      </c>
+      <c r="B14" s="94"/>
       <c r="C14" s="95"/>
       <c r="D14" s="17" t="s">
         <v>38</v>
@@ -3858,10 +3879,10 @@
       <c r="U14" s="26"/>
     </row>
     <row r="15" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="120" t="s">
-        <v>225</v>
-      </c>
-      <c r="B15" s="101"/>
+      <c r="A15" s="116" t="s">
+        <v>224</v>
+      </c>
+      <c r="B15" s="94"/>
       <c r="C15" s="95" t="s">
         <v>39</v>
       </c>
@@ -3926,10 +3947,10 @@
       <c r="U15" s="26"/>
     </row>
     <row r="16" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="120" t="s">
-        <v>226</v>
-      </c>
-      <c r="B16" s="101"/>
+      <c r="A16" s="116" t="s">
+        <v>225</v>
+      </c>
+      <c r="B16" s="94"/>
       <c r="C16" s="95"/>
       <c r="D16" s="17" t="s">
         <v>41</v>
@@ -3992,10 +4013,10 @@
       <c r="U16" s="26"/>
     </row>
     <row r="17" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="120" t="s">
-        <v>227</v>
-      </c>
-      <c r="B17" s="101"/>
+      <c r="A17" s="116" t="s">
+        <v>226</v>
+      </c>
+      <c r="B17" s="94"/>
       <c r="C17" s="95"/>
       <c r="D17" s="17" t="s">
         <v>42</v>
@@ -4058,10 +4079,10 @@
       <c r="U17" s="26"/>
     </row>
     <row r="18" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="120" t="s">
-        <v>228</v>
-      </c>
-      <c r="B18" s="101"/>
+      <c r="A18" s="116" t="s">
+        <v>227</v>
+      </c>
+      <c r="B18" s="94"/>
       <c r="C18" s="95"/>
       <c r="D18" s="17" t="s">
         <v>43</v>
@@ -4124,10 +4145,10 @@
       <c r="U18" s="26"/>
     </row>
     <row r="19" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="120" t="s">
-        <v>229</v>
-      </c>
-      <c r="B19" s="101"/>
+      <c r="A19" s="116" t="s">
+        <v>228</v>
+      </c>
+      <c r="B19" s="94"/>
       <c r="C19" s="95"/>
       <c r="D19" s="17" t="s">
         <v>44</v>
@@ -4190,10 +4211,10 @@
       <c r="U19" s="26"/>
     </row>
     <row r="20" spans="1:21" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="120" t="s">
-        <v>230</v>
-      </c>
-      <c r="B20" s="101"/>
+      <c r="A20" s="116" t="s">
+        <v>229</v>
+      </c>
+      <c r="B20" s="94"/>
       <c r="C20" s="95" t="s">
         <v>45</v>
       </c>
@@ -4258,10 +4279,10 @@
       <c r="U20" s="26"/>
     </row>
     <row r="21" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="120" t="s">
-        <v>231</v>
-      </c>
-      <c r="B21" s="101"/>
+      <c r="A21" s="116" t="s">
+        <v>230</v>
+      </c>
+      <c r="B21" s="94"/>
       <c r="C21" s="95"/>
       <c r="D21" s="95" t="s">
         <v>47</v>
@@ -4326,10 +4347,10 @@
       <c r="U21" s="26"/>
     </row>
     <row r="22" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="120" t="s">
-        <v>232</v>
-      </c>
-      <c r="B22" s="101"/>
+      <c r="A22" s="116" t="s">
+        <v>231</v>
+      </c>
+      <c r="B22" s="94"/>
       <c r="C22" s="95"/>
       <c r="D22" s="95"/>
       <c r="E22" s="2" t="s">
@@ -4392,10 +4413,10 @@
       <c r="U22" s="26"/>
     </row>
     <row r="23" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="120" t="s">
-        <v>233</v>
-      </c>
-      <c r="B23" s="101"/>
+      <c r="A23" s="116" t="s">
+        <v>232</v>
+      </c>
+      <c r="B23" s="94"/>
       <c r="C23" s="95"/>
       <c r="D23" s="95"/>
       <c r="E23" s="2" t="s">
@@ -4458,10 +4479,10 @@
       <c r="U23" s="26"/>
     </row>
     <row r="24" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="120" t="s">
-        <v>234</v>
-      </c>
-      <c r="B24" s="101"/>
+      <c r="A24" s="116" t="s">
+        <v>233</v>
+      </c>
+      <c r="B24" s="94"/>
       <c r="C24" s="95" t="s">
         <v>51</v>
       </c>
@@ -4528,10 +4549,10 @@
       <c r="U24" s="26"/>
     </row>
     <row r="25" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="120" t="s">
-        <v>235</v>
-      </c>
-      <c r="B25" s="101"/>
+      <c r="A25" s="116" t="s">
+        <v>234</v>
+      </c>
+      <c r="B25" s="94"/>
       <c r="C25" s="95"/>
       <c r="D25" s="95"/>
       <c r="E25" s="2" t="s">
@@ -4594,10 +4615,10 @@
       <c r="U25" s="26"/>
     </row>
     <row r="26" spans="1:21" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="120" t="s">
-        <v>236</v>
-      </c>
-      <c r="B26" s="101"/>
+      <c r="A26" s="116" t="s">
+        <v>235</v>
+      </c>
+      <c r="B26" s="94"/>
       <c r="C26" s="95"/>
       <c r="D26" s="95"/>
       <c r="E26" s="2" t="s">
@@ -4660,10 +4681,10 @@
       <c r="U26" s="26"/>
     </row>
     <row r="27" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="120" t="s">
-        <v>237</v>
-      </c>
-      <c r="B27" s="101"/>
+      <c r="A27" s="116" t="s">
+        <v>236</v>
+      </c>
+      <c r="B27" s="94"/>
       <c r="C27" s="95"/>
       <c r="D27" s="95" t="s">
         <v>54</v>
@@ -4728,10 +4749,10 @@
       <c r="U27" s="26"/>
     </row>
     <row r="28" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="120" t="s">
-        <v>238</v>
-      </c>
-      <c r="B28" s="101"/>
+      <c r="A28" s="116" t="s">
+        <v>237</v>
+      </c>
+      <c r="B28" s="94"/>
       <c r="C28" s="95"/>
       <c r="D28" s="95"/>
       <c r="E28" s="2" t="s">
@@ -4794,10 +4815,10 @@
       <c r="U28" s="26"/>
     </row>
     <row r="29" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="120" t="s">
-        <v>239</v>
-      </c>
-      <c r="B29" s="101"/>
+      <c r="A29" s="116" t="s">
+        <v>238</v>
+      </c>
+      <c r="B29" s="94"/>
       <c r="C29" s="95" t="s">
         <v>55</v>
       </c>
@@ -4864,10 +4885,10 @@
       <c r="U29" s="26"/>
     </row>
     <row r="30" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="120" t="s">
-        <v>240</v>
-      </c>
-      <c r="B30" s="101"/>
+      <c r="A30" s="116" t="s">
+        <v>239</v>
+      </c>
+      <c r="B30" s="94"/>
       <c r="C30" s="95"/>
       <c r="D30" s="95"/>
       <c r="E30" s="2" t="s">
@@ -4930,10 +4951,10 @@
       <c r="U30" s="26"/>
     </row>
     <row r="31" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="120" t="s">
-        <v>241</v>
-      </c>
-      <c r="B31" s="101"/>
+      <c r="A31" s="116" t="s">
+        <v>240</v>
+      </c>
+      <c r="B31" s="94"/>
       <c r="C31" s="95"/>
       <c r="D31" s="95"/>
       <c r="E31" s="2" t="s">
@@ -4996,12 +5017,12 @@
       <c r="U31" s="26"/>
     </row>
     <row r="32" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="120" t="s">
-        <v>242</v>
-      </c>
-      <c r="B32" s="101"/>
+      <c r="A32" s="116" t="s">
+        <v>241</v>
+      </c>
+      <c r="B32" s="94"/>
       <c r="C32" s="95"/>
-      <c r="D32" s="97" t="s">
+      <c r="D32" s="100" t="s">
         <v>58</v>
       </c>
       <c r="E32" s="17" t="s">
@@ -5064,12 +5085,12 @@
       <c r="U32" s="26"/>
     </row>
     <row r="33" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="120" t="s">
-        <v>243</v>
-      </c>
-      <c r="B33" s="101"/>
+      <c r="A33" s="116" t="s">
+        <v>242</v>
+      </c>
+      <c r="B33" s="94"/>
       <c r="C33" s="95"/>
-      <c r="D33" s="97"/>
+      <c r="D33" s="100"/>
       <c r="E33" s="2" t="s">
         <v>29</v>
       </c>
@@ -5130,12 +5151,12 @@
       <c r="U33" s="26"/>
     </row>
     <row r="34" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="120" t="s">
-        <v>244</v>
-      </c>
-      <c r="B34" s="101"/>
+      <c r="A34" s="116" t="s">
+        <v>243</v>
+      </c>
+      <c r="B34" s="94"/>
       <c r="C34" s="95"/>
-      <c r="D34" s="97"/>
+      <c r="D34" s="100"/>
       <c r="E34" s="2" t="s">
         <v>35</v>
       </c>
@@ -5196,10 +5217,10 @@
       <c r="U34" s="26"/>
     </row>
     <row r="35" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="120" t="s">
-        <v>245</v>
-      </c>
-      <c r="B35" s="101"/>
+      <c r="A35" s="116" t="s">
+        <v>244</v>
+      </c>
+      <c r="B35" s="94"/>
       <c r="C35" s="95" t="s">
         <v>59</v>
       </c>
@@ -5266,10 +5287,10 @@
       <c r="U35" s="26"/>
     </row>
     <row r="36" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="120" t="s">
-        <v>246</v>
-      </c>
-      <c r="B36" s="101"/>
+      <c r="A36" s="116" t="s">
+        <v>245</v>
+      </c>
+      <c r="B36" s="94"/>
       <c r="C36" s="95"/>
       <c r="D36" s="95"/>
       <c r="E36" s="2" t="s">
@@ -5332,16 +5353,16 @@
       <c r="U36" s="26"/>
     </row>
     <row r="37" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A37" s="120" t="s">
-        <v>247</v>
-      </c>
-      <c r="B37" s="101" t="s">
+      <c r="A37" s="116" t="s">
+        <v>246</v>
+      </c>
+      <c r="B37" s="94" t="s">
         <v>63</v>
       </c>
       <c r="C37" s="95" t="s">
         <v>64</v>
       </c>
-      <c r="D37" s="97" t="s">
+      <c r="D37" s="100" t="s">
         <v>65</v>
       </c>
       <c r="E37" s="17" t="s">
@@ -5404,12 +5425,12 @@
       <c r="U37" s="26"/>
     </row>
     <row r="38" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A38" s="120" t="s">
-        <v>248</v>
-      </c>
-      <c r="B38" s="101"/>
+      <c r="A38" s="116" t="s">
+        <v>247</v>
+      </c>
+      <c r="B38" s="94"/>
       <c r="C38" s="95"/>
-      <c r="D38" s="97"/>
+      <c r="D38" s="100"/>
       <c r="E38" s="2" t="s">
         <v>67</v>
       </c>
@@ -5470,10 +5491,10 @@
       <c r="U38" s="26"/>
     </row>
     <row r="39" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A39" s="120" t="s">
-        <v>249</v>
-      </c>
-      <c r="B39" s="101"/>
+      <c r="A39" s="116" t="s">
+        <v>248</v>
+      </c>
+      <c r="B39" s="94"/>
       <c r="C39" s="95"/>
       <c r="D39" s="17" t="s">
         <v>68</v>
@@ -5536,10 +5557,10 @@
       <c r="U39" s="26"/>
     </row>
     <row r="40" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A40" s="120" t="s">
-        <v>250</v>
-      </c>
-      <c r="B40" s="101"/>
+      <c r="A40" s="116" t="s">
+        <v>249</v>
+      </c>
+      <c r="B40" s="94"/>
       <c r="C40" s="95"/>
       <c r="D40" s="2" t="s">
         <v>69</v>
@@ -5602,10 +5623,10 @@
       <c r="U40" s="26"/>
     </row>
     <row r="41" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A41" s="120" t="s">
-        <v>251</v>
-      </c>
-      <c r="B41" s="101"/>
+      <c r="A41" s="116" t="s">
+        <v>250</v>
+      </c>
+      <c r="B41" s="94"/>
       <c r="C41" s="95"/>
       <c r="D41" s="17" t="s">
         <v>70</v>
@@ -5668,10 +5689,10 @@
       <c r="U41" s="26"/>
     </row>
     <row r="42" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A42" s="120" t="s">
-        <v>252</v>
-      </c>
-      <c r="B42" s="101"/>
+      <c r="A42" s="116" t="s">
+        <v>251</v>
+      </c>
+      <c r="B42" s="94"/>
       <c r="C42" s="95" t="s">
         <v>71</v>
       </c>
@@ -5738,10 +5759,10 @@
       <c r="U42" s="26"/>
     </row>
     <row r="43" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A43" s="120" t="s">
-        <v>253</v>
-      </c>
-      <c r="B43" s="101"/>
+      <c r="A43" s="116" t="s">
+        <v>252</v>
+      </c>
+      <c r="B43" s="94"/>
       <c r="C43" s="95"/>
       <c r="D43" s="95"/>
       <c r="E43" s="2" t="s">
@@ -5804,10 +5825,10 @@
       <c r="U43" s="26"/>
     </row>
     <row r="44" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A44" s="120" t="s">
-        <v>254</v>
-      </c>
-      <c r="B44" s="101"/>
+      <c r="A44" s="116" t="s">
+        <v>253</v>
+      </c>
+      <c r="B44" s="94"/>
       <c r="C44" s="95"/>
       <c r="D44" s="95"/>
       <c r="E44" s="2" t="s">
@@ -5870,14 +5891,14 @@
       <c r="U44" s="26"/>
     </row>
     <row r="45" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A45" s="120" t="s">
-        <v>255</v>
-      </c>
-      <c r="B45" s="101"/>
+      <c r="A45" s="116" t="s">
+        <v>254</v>
+      </c>
+      <c r="B45" s="94"/>
       <c r="C45" s="95" t="s">
         <v>76</v>
       </c>
-      <c r="D45" s="97" t="s">
+      <c r="D45" s="100" t="s">
         <v>77</v>
       </c>
       <c r="E45" s="17" t="s">
@@ -5940,12 +5961,12 @@
       <c r="U45" s="26"/>
     </row>
     <row r="46" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A46" s="120" t="s">
-        <v>256</v>
-      </c>
-      <c r="B46" s="101"/>
+      <c r="A46" s="116" t="s">
+        <v>255</v>
+      </c>
+      <c r="B46" s="94"/>
       <c r="C46" s="95"/>
-      <c r="D46" s="97"/>
+      <c r="D46" s="100"/>
       <c r="E46" s="2" t="s">
         <v>78</v>
       </c>
@@ -6006,10 +6027,10 @@
       <c r="U46" s="26"/>
     </row>
     <row r="47" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A47" s="120" t="s">
-        <v>257</v>
-      </c>
-      <c r="B47" s="101"/>
+      <c r="A47" s="116" t="s">
+        <v>256</v>
+      </c>
+      <c r="B47" s="94"/>
       <c r="C47" s="95"/>
       <c r="D47" s="17" t="s">
         <v>79</v>
@@ -6072,10 +6093,10 @@
       <c r="U47" s="26"/>
     </row>
     <row r="48" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A48" s="120" t="s">
-        <v>258</v>
-      </c>
-      <c r="B48" s="101"/>
+      <c r="A48" s="116" t="s">
+        <v>257</v>
+      </c>
+      <c r="B48" s="94"/>
       <c r="C48" s="95"/>
       <c r="D48" s="2" t="s">
         <v>80</v>
@@ -6138,10 +6159,10 @@
       <c r="U48" s="26"/>
     </row>
     <row r="49" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A49" s="120" t="s">
-        <v>259</v>
-      </c>
-      <c r="B49" s="101"/>
+      <c r="A49" s="116" t="s">
+        <v>258</v>
+      </c>
+      <c r="B49" s="94"/>
       <c r="C49" s="95" t="s">
         <v>81</v>
       </c>
@@ -6208,10 +6229,10 @@
       <c r="U49" s="26"/>
     </row>
     <row r="50" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A50" s="120" t="s">
-        <v>260</v>
-      </c>
-      <c r="B50" s="101"/>
+      <c r="A50" s="116" t="s">
+        <v>259</v>
+      </c>
+      <c r="B50" s="94"/>
       <c r="C50" s="95"/>
       <c r="D50" s="95"/>
       <c r="E50" s="2" t="s">
@@ -6274,16 +6295,16 @@
       <c r="U50" s="26"/>
     </row>
     <row r="51" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A51" s="120" t="s">
-        <v>261</v>
-      </c>
-      <c r="B51" s="101" t="s">
+      <c r="A51" s="116" t="s">
+        <v>260</v>
+      </c>
+      <c r="B51" s="94" t="s">
         <v>85</v>
       </c>
-      <c r="C51" s="100" t="s">
+      <c r="C51" s="93" t="s">
         <v>86</v>
       </c>
-      <c r="D51" s="96" t="s">
+      <c r="D51" s="99" t="s">
         <v>87</v>
       </c>
       <c r="E51" s="12" t="s">
@@ -6346,12 +6367,12 @@
       <c r="U51" s="26"/>
     </row>
     <row r="52" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A52" s="120" t="s">
-        <v>262</v>
-      </c>
-      <c r="B52" s="101"/>
-      <c r="C52" s="100"/>
-      <c r="D52" s="96"/>
+      <c r="A52" s="116" t="s">
+        <v>261</v>
+      </c>
+      <c r="B52" s="94"/>
+      <c r="C52" s="93"/>
+      <c r="D52" s="99"/>
       <c r="E52" s="2" t="s">
         <v>89</v>
       </c>
@@ -6412,12 +6433,12 @@
       <c r="U52" s="26"/>
     </row>
     <row r="53" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A53" s="120" t="s">
-        <v>263</v>
-      </c>
-      <c r="B53" s="101"/>
-      <c r="C53" s="100"/>
-      <c r="D53" s="96"/>
+      <c r="A53" s="116" t="s">
+        <v>262</v>
+      </c>
+      <c r="B53" s="94"/>
+      <c r="C53" s="93"/>
+      <c r="D53" s="99"/>
       <c r="E53" s="2" t="s">
         <v>90</v>
       </c>
@@ -6478,12 +6499,12 @@
       <c r="U53" s="26"/>
     </row>
     <row r="54" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A54" s="120" t="s">
-        <v>264</v>
-      </c>
-      <c r="B54" s="101"/>
-      <c r="C54" s="100"/>
-      <c r="D54" s="96"/>
+      <c r="A54" s="116" t="s">
+        <v>263</v>
+      </c>
+      <c r="B54" s="94"/>
+      <c r="C54" s="93"/>
+      <c r="D54" s="99"/>
       <c r="E54" s="2" t="s">
         <v>91</v>
       </c>
@@ -6544,12 +6565,12 @@
       <c r="U54" s="26"/>
     </row>
     <row r="55" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A55" s="120" t="s">
-        <v>265</v>
-      </c>
-      <c r="B55" s="101"/>
-      <c r="C55" s="100"/>
-      <c r="D55" s="96"/>
+      <c r="A55" s="116" t="s">
+        <v>264</v>
+      </c>
+      <c r="B55" s="94"/>
+      <c r="C55" s="93"/>
+      <c r="D55" s="99"/>
       <c r="E55" s="2" t="s">
         <v>92</v>
       </c>
@@ -6616,14 +6637,14 @@
       </c>
     </row>
     <row r="56" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A56" s="120" t="s">
-        <v>266</v>
-      </c>
-      <c r="B56" s="101"/>
-      <c r="C56" s="100" t="s">
+      <c r="A56" s="116" t="s">
+        <v>265</v>
+      </c>
+      <c r="B56" s="94"/>
+      <c r="C56" s="93" t="s">
         <v>94</v>
       </c>
-      <c r="D56" s="96" t="s">
+      <c r="D56" s="99" t="s">
         <v>95</v>
       </c>
       <c r="E56" s="12" t="s">
@@ -6686,12 +6707,12 @@
       <c r="U56" s="26"/>
     </row>
     <row r="57" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A57" s="120" t="s">
-        <v>267</v>
-      </c>
-      <c r="B57" s="101"/>
-      <c r="C57" s="100"/>
-      <c r="D57" s="96"/>
+      <c r="A57" s="116" t="s">
+        <v>266</v>
+      </c>
+      <c r="B57" s="94"/>
+      <c r="C57" s="93"/>
+      <c r="D57" s="99"/>
       <c r="E57" s="15" t="s">
         <v>96</v>
       </c>
@@ -6752,12 +6773,12 @@
       <c r="U57" s="26"/>
     </row>
     <row r="58" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A58" s="120" t="s">
-        <v>268</v>
-      </c>
-      <c r="B58" s="101"/>
-      <c r="C58" s="100"/>
-      <c r="D58" s="96"/>
+      <c r="A58" s="116" t="s">
+        <v>267</v>
+      </c>
+      <c r="B58" s="94"/>
+      <c r="C58" s="93"/>
+      <c r="D58" s="99"/>
       <c r="E58" s="2" t="s">
         <v>97</v>
       </c>
@@ -6818,12 +6839,12 @@
       <c r="U58" s="26"/>
     </row>
     <row r="59" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A59" s="120" t="s">
-        <v>269</v>
-      </c>
-      <c r="B59" s="101"/>
-      <c r="C59" s="100"/>
-      <c r="D59" s="96"/>
+      <c r="A59" s="116" t="s">
+        <v>268</v>
+      </c>
+      <c r="B59" s="94"/>
+      <c r="C59" s="93"/>
+      <c r="D59" s="99"/>
       <c r="E59" s="2" t="s">
         <v>98</v>
       </c>
@@ -6884,12 +6905,12 @@
       <c r="U59" s="26"/>
     </row>
     <row r="60" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A60" s="120" t="s">
-        <v>270</v>
-      </c>
-      <c r="B60" s="101"/>
-      <c r="C60" s="100"/>
-      <c r="D60" s="96"/>
+      <c r="A60" s="116" t="s">
+        <v>269</v>
+      </c>
+      <c r="B60" s="94"/>
+      <c r="C60" s="93"/>
+      <c r="D60" s="99"/>
       <c r="E60" s="2" t="s">
         <v>99</v>
       </c>
@@ -6950,12 +6971,12 @@
       <c r="U60" s="26"/>
     </row>
     <row r="61" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A61" s="120" t="s">
-        <v>271</v>
-      </c>
-      <c r="B61" s="101"/>
-      <c r="C61" s="100"/>
-      <c r="D61" s="96"/>
+      <c r="A61" s="116" t="s">
+        <v>270</v>
+      </c>
+      <c r="B61" s="94"/>
+      <c r="C61" s="93"/>
+      <c r="D61" s="99"/>
       <c r="E61" s="2" t="s">
         <v>100</v>
       </c>
@@ -7022,14 +7043,14 @@
       </c>
     </row>
     <row r="62" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A62" s="120" t="s">
-        <v>272</v>
-      </c>
-      <c r="B62" s="101"/>
-      <c r="C62" s="100" t="s">
+      <c r="A62" s="116" t="s">
+        <v>271</v>
+      </c>
+      <c r="B62" s="94"/>
+      <c r="C62" s="93" t="s">
         <v>101</v>
       </c>
-      <c r="D62" s="96" t="s">
+      <c r="D62" s="99" t="s">
         <v>102</v>
       </c>
       <c r="E62" s="12" t="s">
@@ -7092,12 +7113,12 @@
       <c r="U62" s="26"/>
     </row>
     <row r="63" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A63" s="120" t="s">
-        <v>273</v>
-      </c>
-      <c r="B63" s="101"/>
-      <c r="C63" s="100"/>
-      <c r="D63" s="96"/>
+      <c r="A63" s="116" t="s">
+        <v>272</v>
+      </c>
+      <c r="B63" s="94"/>
+      <c r="C63" s="93"/>
+      <c r="D63" s="99"/>
       <c r="E63" s="2" t="s">
         <v>103</v>
       </c>
@@ -7158,18 +7179,16 @@
       <c r="U63" s="26"/>
     </row>
     <row r="64" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A64" s="120" t="s">
-        <v>274</v>
-      </c>
-      <c r="B64" s="101"/>
-      <c r="C64" s="100"/>
-      <c r="D64" s="96"/>
+      <c r="A64" s="116" t="s">
+        <v>273</v>
+      </c>
+      <c r="B64" s="94"/>
+      <c r="C64" s="93"/>
+      <c r="D64" s="99"/>
       <c r="E64" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="F64" s="27" t="s">
-        <v>93</v>
-      </c>
+        <v>293</v>
+      </c>
+      <c r="F64" s="25"/>
       <c r="G64" s="61">
         <f t="shared" si="13"/>
         <v>0</v>
@@ -7182,41 +7201,41 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J64" s="59" t="str">
+      <c r="J64" s="59">
         <f t="shared" si="3"/>
-        <v>NA</v>
-      </c>
-      <c r="K64" s="59" t="str">
+        <v>0</v>
+      </c>
+      <c r="K64" s="59">
         <f t="shared" si="4"/>
-        <v>NA</v>
-      </c>
-      <c r="L64" s="59" t="str">
+        <v>0</v>
+      </c>
+      <c r="L64" s="59">
         <f t="shared" si="5"/>
-        <v>NA</v>
+        <v>0</v>
       </c>
       <c r="M64" s="59">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="N64" s="83" t="str">
+      <c r="N64" s="83">
         <f t="shared" si="7"/>
-        <v>NA</v>
-      </c>
-      <c r="O64" s="83" t="str">
+        <v>0</v>
+      </c>
+      <c r="O64" s="83">
         <f t="shared" si="8"/>
-        <v>NA</v>
-      </c>
-      <c r="P64" s="83" t="str">
+        <v>0</v>
+      </c>
+      <c r="P64" s="83">
         <f t="shared" si="9"/>
-        <v>NA</v>
-      </c>
-      <c r="Q64" s="83" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q64" s="83">
         <f t="shared" si="10"/>
-        <v>NA</v>
-      </c>
-      <c r="R64" s="83" t="str">
+        <v>0</v>
+      </c>
+      <c r="R64" s="83">
         <f t="shared" si="11"/>
-        <v>NA</v>
+        <v>0</v>
       </c>
       <c r="S64" s="59">
         <f t="shared" si="12"/>
@@ -7230,14 +7249,14 @@
       </c>
     </row>
     <row r="65" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A65" s="120" t="s">
-        <v>275</v>
-      </c>
-      <c r="B65" s="101"/>
-      <c r="C65" s="100"/>
-      <c r="D65" s="96"/>
+      <c r="A65" s="116" t="s">
+        <v>274</v>
+      </c>
+      <c r="B65" s="94"/>
+      <c r="C65" s="93"/>
+      <c r="D65" s="99"/>
       <c r="E65" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F65" s="27" t="s">
         <v>93</v>
@@ -7302,17 +7321,17 @@
       </c>
     </row>
     <row r="66" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="120" t="s">
-        <v>276</v>
-      </c>
-      <c r="B66" s="88" t="s">
+      <c r="A66" s="116" t="s">
+        <v>275</v>
+      </c>
+      <c r="B66" s="121" t="s">
+        <v>105</v>
+      </c>
+      <c r="C66" s="93" t="s">
         <v>106</v>
       </c>
-      <c r="C66" s="100" t="s">
+      <c r="D66" s="99" t="s">
         <v>107</v>
-      </c>
-      <c r="D66" s="96" t="s">
-        <v>108</v>
       </c>
       <c r="E66" s="12" t="s">
         <v>28</v>
@@ -7374,14 +7393,14 @@
       <c r="U66" s="26"/>
     </row>
     <row r="67" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A67" s="120" t="s">
-        <v>277</v>
-      </c>
-      <c r="B67" s="89"/>
-      <c r="C67" s="100"/>
-      <c r="D67" s="96"/>
+      <c r="A67" s="116" t="s">
+        <v>276</v>
+      </c>
+      <c r="B67" s="122"/>
+      <c r="C67" s="93"/>
+      <c r="D67" s="99"/>
       <c r="E67" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F67" s="25"/>
       <c r="G67" s="61">
@@ -7440,14 +7459,14 @@
       <c r="U67" s="26"/>
     </row>
     <row r="68" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A68" s="120" t="s">
-        <v>278</v>
-      </c>
-      <c r="B68" s="89"/>
-      <c r="C68" s="100"/>
-      <c r="D68" s="96"/>
+      <c r="A68" s="116" t="s">
+        <v>277</v>
+      </c>
+      <c r="B68" s="122"/>
+      <c r="C68" s="93"/>
+      <c r="D68" s="99"/>
       <c r="E68" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F68" s="27" t="s">
         <v>93</v>
@@ -7512,18 +7531,18 @@
       </c>
     </row>
     <row r="69" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A69" s="120" t="s">
-        <v>279</v>
-      </c>
-      <c r="B69" s="89"/>
-      <c r="C69" s="100" t="s">
+      <c r="A69" s="116" t="s">
+        <v>278</v>
+      </c>
+      <c r="B69" s="122"/>
+      <c r="C69" s="93" t="s">
+        <v>110</v>
+      </c>
+      <c r="D69" s="70" t="s">
         <v>111</v>
       </c>
-      <c r="D69" s="70" t="s">
+      <c r="E69" s="85" t="s">
         <v>112</v>
-      </c>
-      <c r="E69" s="85" t="s">
-        <v>113</v>
       </c>
       <c r="F69" s="25"/>
       <c r="G69" s="61">
@@ -7582,16 +7601,16 @@
       <c r="U69" s="26"/>
     </row>
     <row r="70" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A70" s="120" t="s">
-        <v>280</v>
-      </c>
-      <c r="B70" s="89"/>
-      <c r="C70" s="100"/>
+      <c r="A70" s="116" t="s">
+        <v>279</v>
+      </c>
+      <c r="B70" s="122"/>
+      <c r="C70" s="93"/>
       <c r="D70" s="70" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E70" s="85" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F70" s="25"/>
       <c r="G70" s="61">
@@ -7650,13 +7669,13 @@
       <c r="U70" s="26"/>
     </row>
     <row r="71" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A71" s="120" t="s">
-        <v>281</v>
-      </c>
-      <c r="B71" s="89"/>
-      <c r="C71" s="100"/>
+      <c r="A71" s="116" t="s">
+        <v>280</v>
+      </c>
+      <c r="B71" s="122"/>
+      <c r="C71" s="93"/>
       <c r="D71" s="15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E71" s="16"/>
       <c r="F71" s="25"/>
@@ -7716,15 +7735,15 @@
       <c r="U71" s="26"/>
     </row>
     <row r="72" spans="1:21" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A72" s="120" t="s">
-        <v>282</v>
-      </c>
-      <c r="B72" s="89"/>
-      <c r="C72" s="100" t="s">
+      <c r="A72" s="116" t="s">
+        <v>281</v>
+      </c>
+      <c r="B72" s="122"/>
+      <c r="C72" s="93" t="s">
+        <v>115</v>
+      </c>
+      <c r="D72" s="15" t="s">
         <v>116</v>
-      </c>
-      <c r="D72" s="15" t="s">
-        <v>117</v>
       </c>
       <c r="E72" s="16"/>
       <c r="F72" s="25"/>
@@ -7784,13 +7803,13 @@
       <c r="U72" s="26"/>
     </row>
     <row r="73" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A73" s="120" t="s">
-        <v>283</v>
-      </c>
-      <c r="B73" s="89"/>
-      <c r="C73" s="100"/>
+      <c r="A73" s="116" t="s">
+        <v>282</v>
+      </c>
+      <c r="B73" s="122"/>
+      <c r="C73" s="93"/>
       <c r="D73" s="63" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E73" s="67"/>
       <c r="F73" s="25"/>
@@ -7850,13 +7869,13 @@
       <c r="U73" s="26"/>
     </row>
     <row r="74" spans="1:21" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A74" s="120" t="s">
-        <v>284</v>
-      </c>
-      <c r="B74" s="89"/>
-      <c r="C74" s="100"/>
+      <c r="A74" s="116" t="s">
+        <v>283</v>
+      </c>
+      <c r="B74" s="122"/>
+      <c r="C74" s="93"/>
       <c r="D74" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E74" s="16"/>
       <c r="F74" s="25"/>
@@ -7916,15 +7935,15 @@
       <c r="U74" s="26"/>
     </row>
     <row r="75" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A75" s="120" t="s">
-        <v>285</v>
-      </c>
-      <c r="B75" s="89"/>
-      <c r="C75" s="102" t="s">
+      <c r="A75" s="116" t="s">
+        <v>284</v>
+      </c>
+      <c r="B75" s="122"/>
+      <c r="C75" s="92" t="s">
+        <v>119</v>
+      </c>
+      <c r="D75" s="11" t="s">
         <v>120</v>
-      </c>
-      <c r="D75" s="11" t="s">
-        <v>121</v>
       </c>
       <c r="E75" s="14"/>
       <c r="F75" s="25"/>
@@ -7984,13 +8003,13 @@
       <c r="U75" s="26"/>
     </row>
     <row r="76" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A76" s="120" t="s">
-        <v>286</v>
-      </c>
-      <c r="B76" s="89"/>
-      <c r="C76" s="102"/>
+      <c r="A76" s="116" t="s">
+        <v>285</v>
+      </c>
+      <c r="B76" s="122"/>
+      <c r="C76" s="92"/>
       <c r="D76" s="11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E76" s="14"/>
       <c r="F76" s="25"/>
@@ -8050,13 +8069,13 @@
       <c r="U76" s="26"/>
     </row>
     <row r="77" spans="1:21" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A77" s="120" t="s">
-        <v>287</v>
-      </c>
-      <c r="B77" s="89"/>
-      <c r="C77" s="102"/>
+      <c r="A77" s="116" t="s">
+        <v>286</v>
+      </c>
+      <c r="B77" s="122"/>
+      <c r="C77" s="92"/>
       <c r="D77" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E77" s="14"/>
       <c r="F77" s="25"/>
@@ -8116,15 +8135,15 @@
       <c r="U77" s="26"/>
     </row>
     <row r="78" spans="1:21" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A78" s="120" t="s">
-        <v>288</v>
-      </c>
-      <c r="B78" s="89"/>
+      <c r="A78" s="116" t="s">
+        <v>287</v>
+      </c>
+      <c r="B78" s="122"/>
       <c r="C78" s="64" t="s">
+        <v>123</v>
+      </c>
+      <c r="D78" s="65" t="s">
         <v>124</v>
-      </c>
-      <c r="D78" s="65" t="s">
-        <v>125</v>
       </c>
       <c r="E78" s="66"/>
       <c r="F78" s="25"/>
@@ -8184,15 +8203,15 @@
       <c r="U78" s="26"/>
     </row>
     <row r="79" spans="1:21" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A79" s="120" t="s">
-        <v>289</v>
-      </c>
-      <c r="B79" s="89"/>
+      <c r="A79" s="116" t="s">
+        <v>288</v>
+      </c>
+      <c r="B79" s="122"/>
       <c r="C79" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="D79" s="11" t="s">
         <v>126</v>
-      </c>
-      <c r="D79" s="11" t="s">
-        <v>127</v>
       </c>
       <c r="E79" s="14"/>
       <c r="F79" s="25"/>
@@ -8252,15 +8271,15 @@
       <c r="U79" s="26"/>
     </row>
     <row r="80" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A80" s="120" t="s">
-        <v>290</v>
-      </c>
-      <c r="B80" s="89"/>
-      <c r="C80" s="86" t="s">
+      <c r="A80" s="116" t="s">
+        <v>289</v>
+      </c>
+      <c r="B80" s="122"/>
+      <c r="C80" s="124" t="s">
+        <v>127</v>
+      </c>
+      <c r="D80" s="11" t="s">
         <v>128</v>
-      </c>
-      <c r="D80" s="11" t="s">
-        <v>129</v>
       </c>
       <c r="E80" s="14"/>
       <c r="F80" s="25"/>
@@ -8320,13 +8339,13 @@
       <c r="U80" s="26"/>
     </row>
     <row r="81" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A81" s="120" t="s">
-        <v>291</v>
-      </c>
-      <c r="B81" s="90"/>
-      <c r="C81" s="87"/>
+      <c r="A81" s="116" t="s">
+        <v>290</v>
+      </c>
+      <c r="B81" s="122"/>
+      <c r="C81" s="125"/>
       <c r="D81" s="11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E81" s="14"/>
       <c r="F81" s="25"/>
@@ -8385,102 +8404,124 @@
       <c r="T81" s="26"/>
       <c r="U81" s="26"/>
     </row>
-    <row r="82" spans="1:21" s="18" customFormat="1" ht="26.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B82" s="91" t="s">
-        <v>131</v>
-      </c>
-      <c r="C82" s="91"/>
-      <c r="D82" s="91"/>
-      <c r="E82" s="91"/>
-      <c r="F82" s="91"/>
-      <c r="G82" s="91"/>
-      <c r="H82" s="91"/>
-      <c r="I82" s="91"/>
-      <c r="J82" s="69">
+    <row r="82" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A82" s="116" t="s">
+        <v>291</v>
+      </c>
+      <c r="B82" s="123"/>
+      <c r="C82" s="126"/>
+      <c r="D82" s="65" t="s">
+        <v>292</v>
+      </c>
+      <c r="E82" s="66"/>
+      <c r="F82" s="117"/>
+      <c r="G82" s="118"/>
+      <c r="H82" s="118"/>
+      <c r="I82" s="118"/>
+      <c r="J82" s="119"/>
+      <c r="K82" s="119"/>
+      <c r="L82" s="119"/>
+      <c r="M82" s="119"/>
+      <c r="N82" s="62"/>
+      <c r="O82" s="62"/>
+      <c r="P82" s="62"/>
+      <c r="Q82" s="62"/>
+      <c r="R82" s="62"/>
+      <c r="S82" s="59"/>
+      <c r="T82" s="120"/>
+      <c r="U82" s="120"/>
+    </row>
+    <row r="83" spans="1:21" s="18" customFormat="1" ht="26.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B83" s="102" t="s">
+        <v>130</v>
+      </c>
+      <c r="C83" s="102"/>
+      <c r="D83" s="102"/>
+      <c r="E83" s="102"/>
+      <c r="F83" s="102"/>
+      <c r="G83" s="102"/>
+      <c r="H83" s="102"/>
+      <c r="I83" s="102"/>
+      <c r="J83" s="69">
         <f>SUM(J5:J81)</f>
         <v>0</v>
       </c>
-      <c r="K82" s="69">
+      <c r="K83" s="69">
         <f>SUM(K5:K81)</f>
         <v>0</v>
       </c>
-      <c r="L82" s="69">
+      <c r="L83" s="69">
         <f>SUM(L5:L81)</f>
         <v>0</v>
       </c>
-      <c r="M82" s="69">
+      <c r="M83" s="69">
         <f>SUM(M5:M81)</f>
         <v>0</v>
       </c>
-      <c r="N82" s="76">
-        <f t="shared" ref="N82:S82" si="27">SUMIF(N5:N81,"&lt;&gt;#N/A")</f>
-        <v>0</v>
-      </c>
-      <c r="O82" s="76">
+      <c r="N83" s="76">
+        <f t="shared" ref="N83:S83" si="27">SUMIF(N5:N81,"&lt;&gt;#N/A")</f>
+        <v>0</v>
+      </c>
+      <c r="O83" s="76">
         <f t="shared" si="27"/>
         <v>0</v>
       </c>
-      <c r="P82" s="76">
+      <c r="P83" s="76">
         <f t="shared" si="27"/>
         <v>0</v>
       </c>
-      <c r="Q82" s="76">
+      <c r="Q83" s="76">
         <f t="shared" si="27"/>
         <v>0</v>
       </c>
-      <c r="R82" s="76">
+      <c r="R83" s="76">
         <f t="shared" si="27"/>
         <v>0</v>
       </c>
-      <c r="S82" s="76">
+      <c r="S83" s="76">
         <f t="shared" si="27"/>
         <v>0</v>
       </c>
-      <c r="T82" s="69"/>
-      <c r="U82" s="69"/>
-    </row>
-    <row r="83" spans="1:21" s="18" customFormat="1" ht="26.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B83" s="92"/>
-      <c r="C83" s="92"/>
-      <c r="D83" s="92"/>
-      <c r="E83" s="92"/>
-      <c r="F83" s="92"/>
-      <c r="G83" s="92"/>
-      <c r="H83" s="92"/>
-      <c r="I83" s="92"/>
-      <c r="S83" s="68"/>
-    </row>
-    <row r="85" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B85" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="C85" s="4"/>
-      <c r="D85" s="4"/>
+      <c r="T83" s="69"/>
+      <c r="U83" s="69"/>
+    </row>
+    <row r="84" spans="1:21" s="18" customFormat="1" ht="26.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B84" s="103"/>
+      <c r="C84" s="103"/>
+      <c r="D84" s="103"/>
+      <c r="E84" s="103"/>
+      <c r="F84" s="103"/>
+      <c r="G84" s="103"/>
+      <c r="H84" s="103"/>
+      <c r="I84" s="103"/>
+      <c r="S84" s="68"/>
     </row>
     <row r="86" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B86" s="4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C86" s="4"/>
       <c r="D86" s="4"/>
     </row>
     <row r="87" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B87" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C87" s="4"/>
       <c r="D87" s="4"/>
-      <c r="M87" s="19"/>
     </row>
     <row r="88" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B88" s="4" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C88" s="4"/>
       <c r="D88" s="4"/>
+      <c r="M88" s="19"/>
     </row>
     <row r="89" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B89" s="4"/>
+      <c r="B89" s="4" t="s">
+        <v>134</v>
+      </c>
       <c r="C89" s="4"/>
       <c r="D89" s="4"/>
     </row>
@@ -8495,58 +8536,58 @@
       <c r="D91" s="4"/>
     </row>
     <row r="92" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B92" s="103" t="s">
+      <c r="B92" s="4"/>
+      <c r="C92" s="4"/>
+      <c r="D92" s="4"/>
+    </row>
+    <row r="93" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B93" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="C92" s="104"/>
-      <c r="D92" s="75" t="s">
+      <c r="C93" s="87"/>
+      <c r="D93" s="75" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="94" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B94" s="88" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="93" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B93" s="105" t="s">
+      <c r="C94" s="89"/>
+      <c r="D94" s="73">
+        <f>COUNTIF(F5:F36, "NA")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B95" s="88" t="s">
         <v>137</v>
       </c>
-      <c r="C93" s="106"/>
-      <c r="D93" s="73">
-        <f>COUNTIF(F5:F36, "NA")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="94" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B94" s="105" t="s">
+      <c r="C95" s="89"/>
+      <c r="D95" s="73">
+        <f>COUNTIF(F37:F50, "NA")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B96" s="88" t="s">
         <v>138</v>
       </c>
-      <c r="C94" s="106"/>
-      <c r="D94" s="73">
-        <f>COUNTIF(F37:F50, "NA")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="95" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B95" s="105" t="s">
+      <c r="C96" s="89"/>
+      <c r="D96" s="73">
+        <f>COUNTIF(F51:F65, "NA")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="97" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B97" s="90" t="s">
         <v>139</v>
       </c>
-      <c r="C95" s="106"/>
-      <c r="D95" s="73">
-        <f>COUNTIF(F51:F65, "NA")</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="96" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B96" s="107" t="s">
-        <v>140</v>
-      </c>
-      <c r="C96" s="108"/>
-      <c r="D96" s="74">
+      <c r="C97" s="91"/>
+      <c r="D97" s="74">
         <f>COUNTIF(F66:F81,"NA")</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="97" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B97" s="4"/>
-      <c r="C97" s="4"/>
-      <c r="D97" s="4"/>
     </row>
     <row r="98" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B98" s="4"/>
@@ -8558,22 +8599,38 @@
       <c r="C99" s="4"/>
       <c r="D99" s="4"/>
     </row>
+    <row r="100" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B100" s="4"/>
+      <c r="C100" s="4"/>
+      <c r="D100" s="4"/>
+    </row>
   </sheetData>
   <mergeCells count="60">
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B92:C92"/>
-    <mergeCell ref="B93:C93"/>
-    <mergeCell ref="B94:C94"/>
-    <mergeCell ref="B95:C95"/>
-    <mergeCell ref="B96:C96"/>
-    <mergeCell ref="C75:C77"/>
-    <mergeCell ref="C66:C68"/>
-    <mergeCell ref="B37:B50"/>
-    <mergeCell ref="B5:B36"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="C20:C23"/>
-    <mergeCell ref="C37:C41"/>
-    <mergeCell ref="C45:C48"/>
+    <mergeCell ref="D32:D34"/>
+    <mergeCell ref="B66:B82"/>
+    <mergeCell ref="C80:C82"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="D21:D23"/>
+    <mergeCell ref="D24:D26"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="D9:D12"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="J3:M3"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="N3:S3"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="D56:D61"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="D42:D44"/>
+    <mergeCell ref="D45:D46"/>
+    <mergeCell ref="D49:D50"/>
+    <mergeCell ref="D51:D55"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="U3:U4"/>
     <mergeCell ref="C72:C74"/>
@@ -8590,36 +8647,25 @@
     <mergeCell ref="C42:C44"/>
     <mergeCell ref="C29:C34"/>
     <mergeCell ref="C24:C28"/>
-    <mergeCell ref="D35:D36"/>
-    <mergeCell ref="D56:D61"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="D42:D44"/>
-    <mergeCell ref="D45:D46"/>
-    <mergeCell ref="D49:D50"/>
-    <mergeCell ref="D51:D55"/>
-    <mergeCell ref="T3:T4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="J3:M3"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="C80:C81"/>
-    <mergeCell ref="B66:B81"/>
-    <mergeCell ref="B82:I82"/>
+    <mergeCell ref="B97:C97"/>
+    <mergeCell ref="C75:C77"/>
+    <mergeCell ref="C66:C68"/>
+    <mergeCell ref="B37:B50"/>
+    <mergeCell ref="B5:B36"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="C20:C23"/>
+    <mergeCell ref="C37:C41"/>
+    <mergeCell ref="C45:C48"/>
     <mergeCell ref="B83:I83"/>
-    <mergeCell ref="N3:S3"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="D21:D23"/>
-    <mergeCell ref="D24:D26"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="D9:D12"/>
+    <mergeCell ref="B84:I84"/>
     <mergeCell ref="D62:D65"/>
     <mergeCell ref="D27:D28"/>
     <mergeCell ref="D29:D31"/>
-    <mergeCell ref="D32:D34"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B93:C93"/>
+    <mergeCell ref="B94:C94"/>
+    <mergeCell ref="B95:C95"/>
+    <mergeCell ref="B96:C96"/>
   </mergeCells>
   <phoneticPr fontId="22" type="noConversion"/>
   <hyperlinks>
@@ -8643,31 +8689,31 @@
           <x14:formula1>
             <xm:f>'Scoring Guideline'!$B$47:$B$49</xm:f>
           </x14:formula1>
-          <xm:sqref>Q5:Q81</xm:sqref>
+          <xm:sqref>Q5:Q82</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data Validation" error="Please see scoring guideline work sheet" xr:uid="{00000000-0002-0000-0000-000001000000}">
           <x14:formula1>
             <xm:f>'Scoring Guideline'!$B$54:$B$56</xm:f>
           </x14:formula1>
-          <xm:sqref>R5:R81</xm:sqref>
+          <xm:sqref>R5:R82</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Input Validation" error="Please see scoring guideline timesheet" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Scoring Guideline'!$B$34:$B$35</xm:f>
           </x14:formula1>
-          <xm:sqref>O5:O81</xm:sqref>
+          <xm:sqref>O5:O82</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Validation Error" error="Please see scoring guideline worksheet" xr:uid="{00000000-0002-0000-0000-000003000000}">
           <x14:formula1>
             <xm:f>'Scoring Guideline'!$B$40:$B$42</xm:f>
           </x14:formula1>
-          <xm:sqref>P5:P81</xm:sqref>
+          <xm:sqref>P5:P82</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000004000000}">
           <x14:formula1>
             <xm:f>'Scoring Guideline'!$B$28:$B$29</xm:f>
           </x14:formula1>
-          <xm:sqref>N5:N81</xm:sqref>
+          <xm:sqref>N5:N82</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -8695,68 +8741,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="36" x14ac:dyDescent="0.55000000000000004">
-      <c r="B1" s="111" t="s">
-        <v>141</v>
-      </c>
-      <c r="C1" s="111"/>
-      <c r="D1" s="111"/>
-      <c r="E1" s="111"/>
-      <c r="F1" s="111"/>
-      <c r="G1" s="111"/>
-      <c r="H1" s="111"/>
-      <c r="I1" s="111"/>
+      <c r="B1" s="106" t="s">
+        <v>140</v>
+      </c>
+      <c r="C1" s="106"/>
+      <c r="D1" s="106"/>
+      <c r="E1" s="106"/>
+      <c r="F1" s="106"/>
+      <c r="G1" s="106"/>
+      <c r="H1" s="106"/>
+      <c r="I1" s="106"/>
     </row>
     <row r="3" spans="2:9" ht="21" hidden="1" x14ac:dyDescent="0.35">
       <c r="B3" s="10" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" ht="37.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="107" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="4" spans="2:9" ht="37.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="112" t="s">
+      <c r="C4" s="107" t="s">
         <v>143</v>
       </c>
-      <c r="C4" s="112" t="s">
+      <c r="D4" s="107"/>
+      <c r="E4" s="107"/>
+      <c r="F4" s="107" t="s">
         <v>144</v>
       </c>
-      <c r="D4" s="112"/>
-      <c r="E4" s="112"/>
-      <c r="F4" s="112" t="s">
+      <c r="G4" s="107"/>
+      <c r="H4" s="107"/>
+      <c r="I4" s="108" t="s">
         <v>145</v>
       </c>
-      <c r="G4" s="112"/>
-      <c r="H4" s="112"/>
-      <c r="I4" s="113" t="s">
+    </row>
+    <row r="5" spans="2:9" ht="34.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="107"/>
+      <c r="C5" s="7" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="5" spans="2:9" ht="34.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="112"/>
-      <c r="C5" s="7" t="s">
+      <c r="D5" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="E5" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="E5" s="9" t="s">
-        <v>149</v>
-      </c>
       <c r="F5" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="H5" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="H5" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="I5" s="113"/>
+      <c r="I5" s="108"/>
     </row>
     <row r="6" spans="2:9" ht="34.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C6" s="29">
-        <f>(32-Input!D93)*3</f>
+        <f>(32-Input!D94)*3</f>
         <v>96</v>
       </c>
       <c r="D6" s="29">
@@ -8768,7 +8814,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="29">
-        <f>(32-Input!D93)*5</f>
+        <f>(32-Input!D94)*5</f>
         <v>160</v>
       </c>
       <c r="G6" s="29">
@@ -8786,10 +8832,10 @@
     </row>
     <row r="7" spans="2:9" ht="34.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C7" s="29">
-        <f>(14-Input!D94)*3</f>
+        <f>(14-Input!D95)*3</f>
         <v>42</v>
       </c>
       <c r="D7" s="29">
@@ -8801,7 +8847,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="29">
-        <f>(14-Input!D94)*5</f>
+        <f>(14-Input!D95)*5</f>
         <v>70</v>
       </c>
       <c r="G7" s="29">
@@ -8819,11 +8865,11 @@
     </row>
     <row r="8" spans="2:9" ht="34.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C8" s="29">
-        <f>(15-Input!D95)*3</f>
-        <v>33</v>
+        <f>(15-Input!D96)*3</f>
+        <v>36</v>
       </c>
       <c r="D8" s="29">
         <f>SUM(Input!M$51:M$65)-Input!M55-Input!M61-Input!M65</f>
@@ -8834,8 +8880,8 @@
         <v>0</v>
       </c>
       <c r="F8" s="29">
-        <f>(15-Input!D95)*5</f>
-        <v>55</v>
+        <f>(15-Input!D96)*5</f>
+        <v>60</v>
       </c>
       <c r="G8" s="29">
         <f>SUM(Input!S$51:S$65)-Input!S55-Input!S61-Input!S65</f>
@@ -8852,10 +8898,10 @@
     </row>
     <row r="9" spans="2:9" ht="34.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C9" s="29">
-        <f>(16-Input!D96)*3</f>
+        <f>(16-Input!D97)*3</f>
         <v>45</v>
       </c>
       <c r="D9" s="29">
@@ -8867,7 +8913,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="29">
-        <f>(16-Input!D96)*5</f>
+        <f>(16-Input!D97)*5</f>
         <v>75</v>
       </c>
       <c r="G9" s="29">
@@ -8885,20 +8931,20 @@
     </row>
     <row r="10" spans="2:9" ht="34.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="C10" s="104" t="s">
         <v>154</v>
       </c>
-      <c r="C10" s="109" t="s">
-        <v>155</v>
-      </c>
-      <c r="D10" s="110"/>
+      <c r="D10" s="105"/>
       <c r="E10" s="20">
         <f>(D6/C6)*25%+(D7/C7)*25%+ (D8/C8)*25% + (D9/C9)*25%</f>
         <v>0</v>
       </c>
-      <c r="F10" s="109" t="s">
-        <v>156</v>
-      </c>
-      <c r="G10" s="110"/>
+      <c r="F10" s="104" t="s">
+        <v>155</v>
+      </c>
+      <c r="G10" s="105"/>
       <c r="H10" s="20">
         <f>(G6/F6)*25%+(G7/F7)*25%+ (G8/F8)*25% + (G9/F9)*25%</f>
         <v>0</v>
@@ -8910,12 +8956,12 @@
     </row>
     <row r="13" spans="2:9" ht="34.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="14" spans="2:9" ht="34.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="34.9" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -8956,12 +9002,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" ht="33.75" x14ac:dyDescent="0.25">
-      <c r="B2" s="117" t="s">
-        <v>159</v>
-      </c>
-      <c r="C2" s="117"/>
-      <c r="D2" s="117"/>
-      <c r="E2" s="117"/>
+      <c r="B2" s="113" t="s">
+        <v>158</v>
+      </c>
+      <c r="C2" s="113"/>
+      <c r="D2" s="113"/>
+      <c r="E2" s="113"/>
     </row>
     <row r="3" spans="2:5" ht="23.25" x14ac:dyDescent="0.25">
       <c r="B3" s="38"/>
@@ -8970,23 +9016,23 @@
       <c r="E3" s="53"/>
     </row>
     <row r="4" spans="2:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="B4" s="118" t="s">
+      <c r="B4" s="112" t="s">
+        <v>159</v>
+      </c>
+      <c r="C4" s="112"/>
+      <c r="D4" s="112"/>
+      <c r="E4" s="112"/>
+    </row>
+    <row r="5" spans="2:5" s="36" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="109" t="s">
         <v>160</v>
       </c>
-      <c r="C4" s="118"/>
-      <c r="D4" s="118"/>
-      <c r="E4" s="118"/>
-    </row>
-    <row r="5" spans="2:5" s="36" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="114" t="s">
+      <c r="C5" s="110"/>
+      <c r="D5" s="50" t="s">
         <v>161</v>
       </c>
-      <c r="C5" s="115"/>
-      <c r="D5" s="50" t="s">
+      <c r="E5" s="51" t="s">
         <v>162</v>
-      </c>
-      <c r="E5" s="51" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="139.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -8994,13 +9040,13 @@
         <v>1</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D6" s="44" t="s">
+        <v>163</v>
+      </c>
+      <c r="E6" s="32" t="s">
         <v>164</v>
-      </c>
-      <c r="E6" s="32" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="7" spans="2:5" ht="31.5" x14ac:dyDescent="0.25">
@@ -9008,38 +9054,38 @@
         <v>0</v>
       </c>
       <c r="C7" s="35" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D7" s="45" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E7" s="54"/>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" s="58" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C8" s="23"/>
       <c r="D8" s="46"/>
     </row>
     <row r="10" spans="2:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="B10" s="116" t="s">
-        <v>168</v>
-      </c>
-      <c r="C10" s="116"/>
-      <c r="D10" s="116"/>
-      <c r="E10" s="116"/>
+      <c r="B10" s="111" t="s">
+        <v>167</v>
+      </c>
+      <c r="C10" s="111"/>
+      <c r="D10" s="111"/>
+      <c r="E10" s="111"/>
     </row>
     <row r="11" spans="2:5" s="36" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="114" t="s">
+      <c r="B11" s="109" t="s">
+        <v>160</v>
+      </c>
+      <c r="C11" s="110"/>
+      <c r="D11" s="50" t="s">
         <v>161</v>
       </c>
-      <c r="C11" s="115"/>
-      <c r="D11" s="50" t="s">
+      <c r="E11" s="51" t="s">
         <v>162</v>
-      </c>
-      <c r="E11" s="51" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="12" spans="2:5" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -9047,13 +9093,13 @@
         <v>1</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D12" s="44" t="s">
+        <v>168</v>
+      </c>
+      <c r="E12" s="32" t="s">
         <v>169</v>
-      </c>
-      <c r="E12" s="32" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="13" spans="2:5" ht="54.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -9061,13 +9107,13 @@
         <v>0.5</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D13" s="44" t="s">
+        <v>170</v>
+      </c>
+      <c r="E13" s="32" t="s">
         <v>171</v>
-      </c>
-      <c r="E13" s="32" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="14" spans="2:5" ht="31.5" x14ac:dyDescent="0.25">
@@ -9075,30 +9121,30 @@
         <v>0</v>
       </c>
       <c r="C14" s="35" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D14" s="45" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E14" s="54"/>
     </row>
     <row r="16" spans="2:5" ht="21" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="47"/>
     </row>
     <row r="17" spans="2:5" s="36" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="114" t="s">
+      <c r="B17" s="109" t="s">
+        <v>160</v>
+      </c>
+      <c r="C17" s="110"/>
+      <c r="D17" s="50" t="s">
         <v>161</v>
       </c>
-      <c r="C17" s="115"/>
-      <c r="D17" s="50" t="s">
+      <c r="E17" s="51" t="s">
         <v>162</v>
-      </c>
-      <c r="E17" s="51" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -9106,13 +9152,13 @@
         <v>1</v>
       </c>
       <c r="C18" s="31" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D18" s="48" t="s">
+        <v>173</v>
+      </c>
+      <c r="E18" s="33" t="s">
         <v>174</v>
-      </c>
-      <c r="E18" s="33" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="37.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -9120,13 +9166,13 @@
         <v>0.5</v>
       </c>
       <c r="C19" s="31" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D19" s="48" t="s">
+        <v>175</v>
+      </c>
+      <c r="E19" s="33" t="s">
         <v>176</v>
-      </c>
-      <c r="E19" s="33" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="20" spans="2:5" ht="45" x14ac:dyDescent="0.25">
@@ -9134,39 +9180,39 @@
         <v>0</v>
       </c>
       <c r="C20" s="35" t="s">
+        <v>160</v>
+      </c>
+      <c r="D20" s="49" t="s">
+        <v>177</v>
+      </c>
+      <c r="E20" s="56"/>
+    </row>
+    <row r="24" spans="2:5" ht="33.75" x14ac:dyDescent="0.25">
+      <c r="B24" s="113" t="s">
+        <v>178</v>
+      </c>
+      <c r="C24" s="113"/>
+      <c r="D24" s="113"/>
+      <c r="E24" s="113"/>
+    </row>
+    <row r="26" spans="2:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="B26" s="111" t="s">
+        <v>179</v>
+      </c>
+      <c r="C26" s="111"/>
+      <c r="D26" s="111"/>
+      <c r="E26" s="111"/>
+    </row>
+    <row r="27" spans="2:5" s="36" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="109" t="s">
+        <v>160</v>
+      </c>
+      <c r="C27" s="110"/>
+      <c r="D27" s="50" t="s">
         <v>161</v>
       </c>
-      <c r="D20" s="49" t="s">
-        <v>178</v>
-      </c>
-      <c r="E20" s="56"/>
-    </row>
-    <row r="24" spans="2:5" ht="33.75" x14ac:dyDescent="0.25">
-      <c r="B24" s="117" t="s">
-        <v>179</v>
-      </c>
-      <c r="C24" s="117"/>
-      <c r="D24" s="117"/>
-      <c r="E24" s="117"/>
-    </row>
-    <row r="26" spans="2:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="B26" s="116" t="s">
-        <v>180</v>
-      </c>
-      <c r="C26" s="116"/>
-      <c r="D26" s="116"/>
-      <c r="E26" s="116"/>
-    </row>
-    <row r="27" spans="2:5" s="36" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="114" t="s">
-        <v>161</v>
-      </c>
-      <c r="C27" s="115"/>
-      <c r="D27" s="50" t="s">
+      <c r="E27" s="51" t="s">
         <v>162</v>
-      </c>
-      <c r="E27" s="51" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="28" spans="2:5" ht="84.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -9174,13 +9220,13 @@
         <v>1</v>
       </c>
       <c r="C28" s="35" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D28" s="48" t="s">
+        <v>180</v>
+      </c>
+      <c r="E28" s="33" t="s">
         <v>181</v>
-      </c>
-      <c r="E28" s="33" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="29" spans="2:5" ht="30" x14ac:dyDescent="0.25">
@@ -9188,10 +9234,10 @@
         <v>0</v>
       </c>
       <c r="C29" s="35" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D29" s="49" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E29" s="56"/>
     </row>
@@ -9202,23 +9248,23 @@
       <c r="E30" s="80"/>
     </row>
     <row r="32" spans="2:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="B32" s="116" t="s">
-        <v>184</v>
-      </c>
-      <c r="C32" s="116"/>
-      <c r="D32" s="116"/>
-      <c r="E32" s="116"/>
+      <c r="B32" s="111" t="s">
+        <v>183</v>
+      </c>
+      <c r="C32" s="111"/>
+      <c r="D32" s="111"/>
+      <c r="E32" s="111"/>
     </row>
     <row r="33" spans="2:5" s="36" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="114" t="s">
+      <c r="B33" s="109" t="s">
+        <v>160</v>
+      </c>
+      <c r="C33" s="110"/>
+      <c r="D33" s="50" t="s">
         <v>161</v>
       </c>
-      <c r="C33" s="115"/>
-      <c r="D33" s="50" t="s">
+      <c r="E33" s="51" t="s">
         <v>162</v>
-      </c>
-      <c r="E33" s="51" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="34" spans="2:5" ht="53.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -9226,13 +9272,13 @@
         <v>1</v>
       </c>
       <c r="C34" s="35" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D34" s="48" t="s">
+        <v>184</v>
+      </c>
+      <c r="E34" s="33" t="s">
         <v>185</v>
-      </c>
-      <c r="E34" s="33" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="35" spans="2:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
@@ -9240,13 +9286,13 @@
         <v>0</v>
       </c>
       <c r="C35" s="35" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D35" s="49" t="s">
+        <v>186</v>
+      </c>
+      <c r="E35" s="57" t="s">
         <v>187</v>
-      </c>
-      <c r="E35" s="57" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.25">
@@ -9256,23 +9302,23 @@
       <c r="E36" s="80"/>
     </row>
     <row r="38" spans="2:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="B38" s="116" t="s">
-        <v>189</v>
-      </c>
-      <c r="C38" s="116"/>
-      <c r="D38" s="116"/>
-      <c r="E38" s="116"/>
+      <c r="B38" s="111" t="s">
+        <v>188</v>
+      </c>
+      <c r="C38" s="111"/>
+      <c r="D38" s="111"/>
+      <c r="E38" s="111"/>
     </row>
     <row r="39" spans="2:5" s="36" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="114" t="s">
+      <c r="B39" s="109" t="s">
+        <v>160</v>
+      </c>
+      <c r="C39" s="110"/>
+      <c r="D39" s="50" t="s">
         <v>161</v>
       </c>
-      <c r="C39" s="115"/>
-      <c r="D39" s="50" t="s">
+      <c r="E39" s="51" t="s">
         <v>162</v>
-      </c>
-      <c r="E39" s="51" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="40" spans="2:5" ht="47.25" x14ac:dyDescent="0.25">
@@ -9280,13 +9326,13 @@
         <v>1</v>
       </c>
       <c r="C40" s="31" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D40" s="44" t="s">
+        <v>189</v>
+      </c>
+      <c r="E40" s="32" t="s">
         <v>190</v>
-      </c>
-      <c r="E40" s="32" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="41" spans="2:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
@@ -9294,13 +9340,13 @@
         <v>0.5</v>
       </c>
       <c r="C41" s="31" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D41" s="44" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E41" s="32" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="42" spans="2:5" ht="47.25" x14ac:dyDescent="0.25">
@@ -9308,13 +9354,13 @@
         <v>0</v>
       </c>
       <c r="C42" s="35" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D42" s="45" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E42" s="34" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.25">
@@ -9324,23 +9370,23 @@
       <c r="E43" s="80"/>
     </row>
     <row r="45" spans="2:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="B45" s="118" t="s">
-        <v>194</v>
-      </c>
-      <c r="C45" s="118"/>
-      <c r="D45" s="118"/>
-      <c r="E45" s="118"/>
+      <c r="B45" s="112" t="s">
+        <v>193</v>
+      </c>
+      <c r="C45" s="112"/>
+      <c r="D45" s="112"/>
+      <c r="E45" s="112"/>
     </row>
     <row r="46" spans="2:5" s="36" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="114" t="s">
+      <c r="B46" s="109" t="s">
+        <v>160</v>
+      </c>
+      <c r="C46" s="110"/>
+      <c r="D46" s="50" t="s">
         <v>161</v>
       </c>
-      <c r="C46" s="115"/>
-      <c r="D46" s="50" t="s">
+      <c r="E46" s="51" t="s">
         <v>162</v>
-      </c>
-      <c r="E46" s="51" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="47" spans="2:5" ht="265.89999999999998" customHeight="1" x14ac:dyDescent="0.25">
@@ -9348,13 +9394,13 @@
         <v>1</v>
       </c>
       <c r="C47" s="31" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D47" s="44" t="s">
+        <v>194</v>
+      </c>
+      <c r="E47" s="32" t="s">
         <v>195</v>
-      </c>
-      <c r="E47" s="32" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="48" spans="2:5" ht="45.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -9362,13 +9408,13 @@
         <v>0.5</v>
       </c>
       <c r="C48" s="31" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D48" s="44" t="s">
+        <v>196</v>
+      </c>
+      <c r="E48" s="32" t="s">
         <v>197</v>
-      </c>
-      <c r="E48" s="32" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="49" spans="2:5" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9376,10 +9422,10 @@
         <v>0</v>
       </c>
       <c r="C49" s="35" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D49" s="45" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E49" s="54"/>
     </row>
@@ -9390,23 +9436,23 @@
       <c r="E50" s="80"/>
     </row>
     <row r="52" spans="2:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="B52" s="118" t="s">
-        <v>200</v>
-      </c>
-      <c r="C52" s="118"/>
-      <c r="D52" s="118"/>
-      <c r="E52" s="118"/>
+      <c r="B52" s="112" t="s">
+        <v>199</v>
+      </c>
+      <c r="C52" s="112"/>
+      <c r="D52" s="112"/>
+      <c r="E52" s="112"/>
     </row>
     <row r="53" spans="2:5" s="36" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="114" t="s">
+      <c r="B53" s="109" t="s">
+        <v>160</v>
+      </c>
+      <c r="C53" s="110"/>
+      <c r="D53" s="50" t="s">
         <v>161</v>
       </c>
-      <c r="C53" s="115"/>
-      <c r="D53" s="50" t="s">
+      <c r="E53" s="51" t="s">
         <v>162</v>
-      </c>
-      <c r="E53" s="51" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="54" spans="2:5" ht="47.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -9414,13 +9460,13 @@
         <v>1</v>
       </c>
       <c r="C54" s="31" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D54" s="48" t="s">
+        <v>200</v>
+      </c>
+      <c r="E54" s="33" t="s">
         <v>201</v>
-      </c>
-      <c r="E54" s="33" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="55" spans="2:5" ht="43.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -9428,13 +9474,13 @@
         <v>0.5</v>
       </c>
       <c r="C55" s="31" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D55" s="48" t="s">
+        <v>202</v>
+      </c>
+      <c r="E55" s="33" t="s">
         <v>203</v>
-      </c>
-      <c r="E55" s="33" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="56" spans="2:5" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -9442,13 +9488,13 @@
         <v>0</v>
       </c>
       <c r="C56" s="35" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D56" s="49" t="s">
+        <v>204</v>
+      </c>
+      <c r="E56" s="37" t="s">
         <v>205</v>
-      </c>
-      <c r="E56" s="37" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.25">
@@ -9459,6 +9505,13 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B24:E24"/>
     <mergeCell ref="B53:C53"/>
     <mergeCell ref="B38:E38"/>
     <mergeCell ref="B45:E45"/>
@@ -9469,13 +9522,6 @@
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B24:E24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="60" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -9489,25 +9535,25 @@
   <sheetData>
     <row r="1" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A1" s="71" t="s">
+        <v>206</v>
+      </c>
+      <c r="B1" s="71" t="s">
         <v>207</v>
       </c>
-      <c r="B1" s="71" t="s">
+      <c r="C1" s="71" t="s">
         <v>208</v>
       </c>
-      <c r="C1" s="71" t="s">
+      <c r="D1" s="71" t="s">
         <v>209</v>
       </c>
-      <c r="D1" s="71" t="s">
+      <c r="E1" s="71" t="s">
         <v>210</v>
       </c>
-      <c r="E1" s="71" t="s">
+      <c r="F1" s="71" t="s">
         <v>211</v>
       </c>
-      <c r="F1" s="71" t="s">
+      <c r="G1" s="71" t="s">
         <v>212</v>
-      </c>
-      <c r="G1" s="71" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -9573,14 +9619,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c60934e2-568b-408c-90a9-1d280ab9521c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="67429372-753f-4bf2-8562-4985ce4a9539" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9839,21 +9883,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c60934e2-568b-408c-90a9-1d280ab9521c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="67429372-753f-4bf2-8562-4985ce4a9539" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5BC44D1-5573-44AE-B196-1A561BD16CB1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D953E4B0-9C71-4486-AD55-F2EC284A4EC0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c60934e2-568b-408c-90a9-1d280ab9521c"/>
-    <ds:schemaRef ds:uri="67429372-753f-4bf2-8562-4985ce4a9539"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9878,9 +9921,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D953E4B0-9C71-4486-AD55-F2EC284A4EC0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5BC44D1-5573-44AE-B196-1A561BD16CB1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c60934e2-568b-408c-90a9-1d280ab9521c"/>
+    <ds:schemaRef ds:uri="67429372-753f-4bf2-8562-4985ce4a9539"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>